<commit_message>
pushing word doc with normalization tables
</commit_message>
<xml_diff>
--- a/module-3/gordon_module3_2.xlsx
+++ b/module-3/gordon_module3_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\csd\csd-310\module-3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAE8FDC-8DBF-4C39-91EC-70FFA20C0ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6891462E-1891-43CD-BD40-6A6BF7149619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4EBE3D19-3CC6-4600-A088-45104FD78424}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4EBE3D19-3CC6-4600-A088-45104FD78424}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
   <si>
     <t>publisher_name</t>
   </si>
@@ -59,9 +59,6 @@
     <t>author_email</t>
   </si>
   <si>
-    <t>publisher_address</t>
-  </si>
-  <si>
     <t>author_first_name</t>
   </si>
   <si>
@@ -74,7 +71,52 @@
     <t>book_isbn</t>
   </si>
   <si>
-    <t>author_address</t>
+    <t>Publisher Table</t>
+  </si>
+  <si>
+    <t>Author Table</t>
+  </si>
+  <si>
+    <t>author_ID</t>
+  </si>
+  <si>
+    <t>Book Table</t>
+  </si>
+  <si>
+    <t>A publisher can publish many books</t>
+  </si>
+  <si>
+    <t>A book can only have one publisher</t>
+  </si>
+  <si>
+    <t>An author can write many books</t>
+  </si>
+  <si>
+    <t>A book can have many authors</t>
+  </si>
+  <si>
+    <t>Book Author Table</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>zip</t>
+  </si>
+  <si>
+    <t>copy</t>
+  </si>
+  <si>
+    <t>Publisher Address Table</t>
+  </si>
+  <si>
+    <t>Author Address Table</t>
   </si>
 </sst>
 </file>
@@ -98,7 +140,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -106,12 +148,93 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,73 +569,432 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56721537-A101-4150-A505-22D6D4E2E89E}">
-  <dimension ref="B3:B14"/>
+  <dimension ref="B1:L34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" customWidth="1"/>
+    <col min="4" max="5" width="17.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" customWidth="1"/>
+    <col min="8" max="8" width="17.88671875" customWidth="1"/>
+    <col min="9" max="11" width="17.77734375" customWidth="1"/>
+    <col min="12" max="12" width="18.109375" customWidth="1"/>
+    <col min="13" max="13" width="17.77734375" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" customWidth="1"/>
+    <col min="15" max="15" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B1" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="8"/>
+    </row>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B3" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="1">
+        <v>2</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B5" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="1">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B6" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="1">
+        <v>4</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B7" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="1">
+        <v>5</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="5"/>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
+      <c r="D10" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
+      <c r="E10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="1">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B12" s="2">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="1">
+        <v>2</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B13" s="2">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="1">
+        <v>3</v>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="2">
+        <v>4</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="1">
+        <v>4</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B15" s="2">
+        <v>5</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="1">
+        <v>5</v>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>11</v>
-      </c>
+      <c r="C19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="G19" s="13"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="H26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="H28" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="H9:L9"/>
+    <mergeCell ref="H1:L1"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B1:D1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>